<commit_message>
Update reports 2026-10-09 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-09.xlsx
+++ b/gex_pivot_levels_2026-10-09.xlsx
@@ -19,8 +19,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -593,37 +593,33 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="2" t="n">
         <v>7774.14</v>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="2" t="n">
         <v>7700</v>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>-$8.69M</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>+$13.99M</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>-$6.95M</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>+$11.19M</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
@@ -639,12 +635,12 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>+$453.89K</t>
+          <t>+$389.04K</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>+$25.96M</t>
+          <t>+$22.25M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -701,12 +697,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>-$9.50M</t>
+          <t>-$8.28M</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>+$15.13M</t>
+          <t>+$13.19M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -734,12 +730,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>-$907.15K</t>
+          <t>-$830.27K</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+$44.07M</t>
+          <t>+$40.33M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -763,12 +759,12 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>+$2.45M</t>
+          <t>+$2.28M</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+$27.02M</t>
+          <t>+$25.12M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -792,12 +788,12 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>+$25.11M</t>
+          <t>+$23.92M</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>+$52.10M</t>
+          <t>+$49.62M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -854,12 +850,12 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>+$1.20M</t>
+          <t>+$1.24M</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>+$36.46M</t>
+          <t>+$37.55M</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -887,12 +883,12 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>+$36.89M</t>
+          <t>+$39.11M</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>+$90.92M</t>
+          <t>+$96.38M</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -920,12 +916,12 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>+$14.83M</t>
+          <t>+$16.22M</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>+$23.09M</t>
+          <t>+$25.25M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -953,12 +949,12 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>+$26.61M</t>
+          <t>+$29.53M</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>+$41.11M</t>
+          <t>+$45.62M</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -986,12 +982,12 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>+$17.78M</t>
+          <t>+$20.40M</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>+$39.48M</t>
+          <t>+$45.28M</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1048,12 +1044,12 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>+$12.91M</t>
+          <t>+$14.57M</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>+$24.50M</t>
+          <t>+$27.66M</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -2963,7 +2959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3014,10 +3010,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>4051.13</v>
+        <v>4084.43</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
@@ -3026,12 +3022,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$1.25M</t>
+          <t>-$1.97M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$1.27M</t>
+          <t>+$2.01M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -3043,109 +3039,109 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>4084.43</v>
+        <v>4118.95</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>368</v>
+        <v>85</v>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>-$7.06M</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>+$7.97M</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>4162.12</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>375</v>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>-$1.95M</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>+$2.00M</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>-$2.61M</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>+$6.79M</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>4095.53</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>369</v>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4184.32</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>377</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>-$172.93K</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>+$237.72K</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>-$164.25K</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>+$4.54M</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>4118.95</v>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>85</v>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>-$7.06M</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>+$7.97M</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>4162.12</v>
+        <v>4195.42</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
@@ -3154,12 +3150,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>-$2.36M</t>
+          <t>-$4.12M</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>+$7.40M</t>
+          <t>+$10.51M</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -3174,66 +3170,66 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>4173.22</v>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>376</v>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="A7" s="5" t="n">
+        <v>4217.62</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>380</v>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>-$120.79K</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>+$1.68M</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>+$3.42M</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>+$14.14M</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>4228.72</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>381</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>+$33.88K</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>+$4.34M</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
-        <v>4195.42</v>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>378</v>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>-$4.91M</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>+$7.11M</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -3241,10 +3237,10 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>4217.62</v>
+        <v>4239.81</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
@@ -3253,12 +3249,12 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>+$1.80M</t>
+          <t>+$9.02M</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>+$11.85M</t>
+          <t>+$11.97M</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -3273,110 +3269,106 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>4228.72</v>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>381</v>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="A10" s="5" t="n">
+        <v>4264.33</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>+$23.46M</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>+$25.39M</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>4273.11</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>385</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>-$329.02K</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>+$3.98M</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>+$3.37M</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>+$4.17M</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>4288.56</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>+$564.05K</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>+$718.62K</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>4239.81</v>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>382</v>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>+$6.81M</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>+$9.19M</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
-        <v>4264.33</v>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>88</v>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>+$23.46M</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>+$25.39M</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>4273.11</v>
+        <v>4328.61</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -3385,12 +3377,12 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>+$2.20M</t>
+          <t>+$1.53M</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$3.15M</t>
+          <t>+$1.56M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -3401,102 +3393,40 @@
       <c r="G13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>4288.56</v>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>88.5</v>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="A14" s="5" t="n">
+        <v>4337.01</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>+$564.05K</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>+$718.62K</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>4328.61</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>390</v>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>+$1.40M</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>+$2.34M</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="n">
-        <v>4337.01</v>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>89.5</v>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>+$7.38M</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>+$7.49M</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G16"/>
+  <autoFilter ref="A1:G14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3508,7 +3438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3748,112 +3678,112 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>7874.14</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>7800</v>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>+$39.11M</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>+$96.38M</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B8" s="5" t="n">
         <v>31213.46</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C8" s="5" t="n">
         <v>750</v>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>-$20.35M</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>+$94.86M</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B9" s="2" t="n">
         <v>7800.07</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C9" s="2" t="n">
         <v>770</v>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>-$20.80M</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>+$94.03M</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>7874.14</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>7800</v>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>+$36.89M</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>+$90.92M</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -3950,12 +3880,12 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>+$25.11M</t>
+          <t>+$23.92M</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>+$52.10M</t>
+          <t>+$49.62M</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -4008,110 +3938,110 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
-        <v>7824.14</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>7750</v>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="B14" s="5" t="n">
+        <v>7884.14</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>7810</v>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>-$907.15K</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>+$44.07M</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr"/>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>+$29.53M</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>+$45.62M</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>7899.14</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>7825</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>+$20.40M</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>+$45.28M</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B16" s="2" t="n">
         <v>31131.26</v>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="C16" s="2" t="n">
         <v>748</v>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>+$12.68M</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>+$42.92M</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>7884.14</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>7810</v>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>+$26.61M</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>+$41.11M</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4124,24 +4054,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>7899.14</v>
+        <v>7824.14</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>7825</v>
+        <v>7750</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>+$17.78M</t>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>-$830.27K</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>+$39.48M</t>
+          <t>+$40.33M</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -4204,12 +4134,12 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>+$1.20M</t>
+          <t>+$1.24M</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>+$36.46M</t>
+          <t>+$37.55M</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -4302,10 +4232,10 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>7834.14</v>
+        <v>7924.14</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>7760</v>
+        <v>7850</v>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
@@ -4314,12 +4244,12 @@
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>+$2.45M</t>
+          <t>+$14.57M</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>+$27.02M</t>
+          <t>+$27.66M</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -4370,28 +4300,28 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>7799.14</v>
+        <v>30802.46</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>7725</v>
+        <v>740</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>+$453.89K</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>-$14.48M</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>+$25.96M</t>
+          <t>+$25.94M</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -4401,35 +4331,35 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>30802.46</v>
+        <v>4264.33</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>740</v>
+        <v>88</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>-$14.48M</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>+$23.46M</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>+$25.94M</t>
+          <t>+$25.39M</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -4439,45 +4369,45 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>7879.14</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>7805</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>+$16.22M</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>+$25.25M</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>4264.33</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>88</v>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>+$23.46M</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>+$25.39M</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4488,10 +4418,10 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>7924.14</v>
+        <v>7834.14</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>7850</v>
+        <v>7760</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
@@ -4500,12 +4430,12 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>+$12.91M</t>
+          <t>+$2.28M</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>+$24.50M</t>
+          <t>+$25.12M</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -4516,40 +4446,40 @@
       <c r="H27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
-        <v>7879.14</v>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>7805</v>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="B28" s="5" t="n">
+        <v>7799.14</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>7725</v>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
-        <is>
-          <t>+$14.83M</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>+$23.09M</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>+$389.04K</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>+$22.25M</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4668,76 +4598,76 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>4217.62</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>380</v>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>+$3.42M</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>+$14.14M</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
+      <c r="B33" s="2" t="n">
         <v>7804.14</v>
       </c>
-      <c r="C32" s="2" t="n">
+      <c r="C33" s="2" t="n">
         <v>7730</v>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>-$9.50M</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>+$15.13M</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>-$8.28M</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>+$13.19M</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n">
-        <v>7774.14</v>
-      </c>
-      <c r="C33" s="5" t="n">
-        <v>7700</v>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>-$8.69M</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>+$13.99M</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4788,10 +4718,10 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>4217.62</v>
+        <v>4239.81</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
@@ -4800,12 +4730,12 @@
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>+$1.80M</t>
+          <t>+$9.02M</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>+$11.85M</t>
+          <t>+$11.97M</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -4860,40 +4790,36 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>30925.76</v>
+        <v>7774.14</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>743</v>
+        <v>7700</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>-$1.71M</t>
+          <t>-$6.95M</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>+$10.28M</t>
+          <t>+$11.19M</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -4902,24 +4828,24 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>4239.81</v>
+        <v>4195.42</v>
       </c>
       <c r="C38" s="5" t="n">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>+$6.81M</t>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>-$4.12M</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>+$9.19M</t>
+          <t>+$10.51M</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
@@ -4929,81 +4855,81 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>30925.76</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>743</v>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>-$1.71M</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>+$10.28M</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
+      <c r="B40" s="2" t="n">
         <v>7940.54</v>
       </c>
-      <c r="C39" s="2" t="n">
+      <c r="C40" s="2" t="n">
         <v>784</v>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="E40" s="9" t="inlineStr">
         <is>
           <t>+$6.93M</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="F40" s="3" t="inlineStr">
         <is>
           <t>+$8.21M</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G40" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="n">
-        <v>4118.95</v>
-      </c>
-      <c r="C40" s="5" t="n">
-        <v>85</v>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>-$7.06M</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>+$7.97M</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -5016,110 +4942,110 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
+        <v>4118.95</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>-$7.06M</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>+$7.97M</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
         <v>4337.01</v>
       </c>
-      <c r="C41" s="5" t="n">
+      <c r="C42" s="5" t="n">
         <v>89.5</v>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E41" s="8" t="inlineStr">
+      <c r="E42" s="8" t="inlineStr">
         <is>
           <t>+$7.38M</t>
         </is>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>+$7.49M</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
+      <c r="G42" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H41" s="6" t="inlineStr">
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B42" s="2" t="n">
+      <c r="B43" s="2" t="n">
         <v>30761.36</v>
       </c>
-      <c r="C42" s="2" t="n">
+      <c r="C43" s="2" t="n">
         <v>739</v>
       </c>
-      <c r="D42" s="3" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>-$567.76K</t>
         </is>
       </c>
-      <c r="F42" s="3" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>+$7.46M</t>
         </is>
       </c>
-      <c r="G42" s="3" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H42" s="3" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="n">
-        <v>4162.12</v>
-      </c>
-      <c r="C43" s="5" t="n">
-        <v>375</v>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="inlineStr">
-        <is>
-          <t>-$2.36M</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr">
-        <is>
-          <t>+$7.40M</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5130,10 +5056,10 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>4195.42</v>
+        <v>4162.12</v>
       </c>
       <c r="C44" s="5" t="n">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
@@ -5142,12 +5068,12 @@
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>-$4.91M</t>
+          <t>-$2.61M</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>+$7.11M</t>
+          <t>+$6.79M</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -5200,114 +5126,118 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>4184.32</v>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>377</v>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>-$164.25K</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>+$4.54M</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B46" s="5" t="n">
+      <c r="B47" s="5" t="n">
         <v>88.23999999999999</v>
       </c>
-      <c r="C46" s="5" t="n">
+      <c r="C47" s="5" t="n">
         <v>144</v>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E46" s="8" t="inlineStr">
+      <c r="E47" s="8" t="inlineStr">
         <is>
           <t>+$2.26M</t>
         </is>
       </c>
-      <c r="F46" s="6" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>+$4.42M</t>
         </is>
       </c>
-      <c r="G46" s="6" t="inlineStr">
+      <c r="G47" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H46" s="6" t="inlineStr">
+      <c r="H47" s="6" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="n">
-        <v>4228.72</v>
-      </c>
-      <c r="C47" s="2" t="n">
-        <v>381</v>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>-$329.02K</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>+$3.98M</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>91.91</v>
+        <v>4228.72</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>150</v>
+        <v>381</v>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>+$2.40M</t>
+          <t>+$33.88K</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>+$3.74M</t>
+          <t>+$4.34M</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -5328,12 +5258,12 @@
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>+$2.20M</t>
+          <t>+$3.37M</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>+$3.15M</t>
+          <t>+$4.17M</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -5350,10 +5280,10 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>92.53</v>
+        <v>91.91</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
@@ -5362,50 +5292,46 @@
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>+$2.48M</t>
+          <t>+$2.40M</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>+$3.13M</t>
+          <t>+$3.74M</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>30555.86</v>
+        <v>92.53</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>734</v>
+        <v>151</v>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>+$464.38K</t>
+          <t>+$2.48M</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>+$2.81M</t>
+          <t>+$3.13M</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -5422,138 +5348,134 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>30555.86</v>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>734</v>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>+$464.38K</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>+$2.81M</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B52" s="2" t="n">
-        <v>4328.61</v>
-      </c>
-      <c r="C52" s="2" t="n">
-        <v>390</v>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
+      <c r="B53" s="2" t="n">
+        <v>4084.43</v>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>368</v>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E52" s="9" t="inlineStr">
-        <is>
-          <t>+$1.40M</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>+$2.34M</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>-$1.97M</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>+$2.01M</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H52" s="3" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="n">
-        <v>4084.43</v>
-      </c>
-      <c r="C53" s="5" t="n">
-        <v>368</v>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>-$1.95M</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>+$2.00M</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>4173.22</v>
+        <v>87.62</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>376</v>
+        <v>143</v>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>-$120.79K</t>
+          <t>-$661.31K</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>+$1.68M</t>
+          <t>+$1.59M</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>87.62</v>
+        <v>4328.61</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>143</v>
+        <v>390</v>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>-$661.31K</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>+$1.53M</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>+$1.59M</t>
+          <t>+$1.56M</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -5602,296 +5524,296 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="n">
-        <v>4051.13</v>
-      </c>
-      <c r="C57" s="2" t="n">
-        <v>365</v>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>-$1.25M</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>+$1.27M</t>
-        </is>
-      </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>85.17</v>
+      </c>
+      <c r="C57" s="5" t="n">
+        <v>139</v>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>-$1.19M</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>+$1.23M</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>89.45999999999999</v>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>146</v>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>+$106.66K</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>+$1.07M</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="n">
+        <v>31088.19</v>
+      </c>
+      <c r="C59" s="5" t="n">
+        <v>30700</v>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>-$632.34K</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>+$1.02M</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>153</v>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>+$145.38K</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>+$894.67K</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H57" s="3" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B58" s="5" t="n">
-        <v>85.17</v>
-      </c>
-      <c r="C58" s="5" t="n">
-        <v>139</v>
-      </c>
-      <c r="D58" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="inlineStr">
-        <is>
-          <t>-$1.19M</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="inlineStr">
-        <is>
-          <t>+$1.23M</t>
-        </is>
-      </c>
-      <c r="G58" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H58" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="n">
-        <v>89.45999999999999</v>
-      </c>
-      <c r="C59" s="2" t="n">
-        <v>146</v>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E59" s="9" t="inlineStr">
-        <is>
-          <t>+$106.66K</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>+$1.07M</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="n">
-        <v>31088.19</v>
-      </c>
-      <c r="C60" s="5" t="n">
-        <v>30700</v>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E60" s="7" t="inlineStr">
-        <is>
-          <t>-$632.34K</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>+$1.02M</t>
-        </is>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>93.75</v>
+        <v>4288.56</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>153</v>
+        <v>88.5</v>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>+$145.38K</t>
+          <t>+$564.05K</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>+$894.67K</t>
+          <t>+$718.62K</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>4288.56</v>
+        <v>31188.19</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>88.5</v>
+        <v>30800</v>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>+$564.05K</t>
+          <t>+$12.90K</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>+$718.62K</t>
+          <t>+$658.15K</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H62" s="3" t="inlineStr">
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n">
+        <v>30988.19</v>
+      </c>
+      <c r="C63" s="5" t="n">
+        <v>30600</v>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>-$475.64K</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>+$608.37K</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B63" s="2" t="n">
-        <v>31188.19</v>
-      </c>
-      <c r="C63" s="2" t="n">
-        <v>30800</v>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
+      <c r="B64" s="2" t="n">
+        <v>31288.19</v>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>30900</v>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E63" s="9" t="inlineStr">
-        <is>
-          <t>+$12.90K</t>
-        </is>
-      </c>
-      <c r="F63" s="3" t="inlineStr">
-        <is>
-          <t>+$658.15K</t>
-        </is>
-      </c>
-      <c r="G63" s="3" t="inlineStr">
+      <c r="E64" s="9" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>+$551.22K</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H63" s="3" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="n">
-        <v>30988.19</v>
-      </c>
-      <c r="C64" s="5" t="n">
-        <v>30600</v>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="inlineStr">
-        <is>
-          <t>-$475.64K</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>+$608.37K</t>
-        </is>
-      </c>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -5900,24 +5822,24 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>31288.19</v>
+        <v>31138.19</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>30900</v>
+        <v>30750</v>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E65" s="9" t="inlineStr">
-        <is>
-          <t>$0</t>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>-$172.06K</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>+$551.22K</t>
+          <t>+$430.16K</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -5928,38 +5850,42 @@
       <c r="H65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+      <c r="A66" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B66" s="2" t="n">
-        <v>31138.19</v>
-      </c>
-      <c r="C66" s="2" t="n">
-        <v>30750</v>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
+      <c r="B66" s="5" t="n">
+        <v>31048.19</v>
+      </c>
+      <c r="C66" s="5" t="n">
+        <v>30660</v>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr">
-        <is>
-          <t>-$172.06K</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>+$430.16K</t>
-        </is>
-      </c>
-      <c r="G66" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H66" s="3" t="inlineStr"/>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>-$327.54K</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>+$407.42K</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
@@ -5968,10 +5894,10 @@
         </is>
       </c>
       <c r="B67" s="5" t="n">
-        <v>31048.19</v>
+        <v>31118.19</v>
       </c>
       <c r="C67" s="5" t="n">
-        <v>30660</v>
+        <v>30730</v>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
@@ -5980,12 +5906,12 @@
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>-$327.54K</t>
+          <t>-$210.78K</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>+$407.42K</t>
+          <t>+$348.43K</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr">
@@ -6006,10 +5932,10 @@
         </is>
       </c>
       <c r="B68" s="5" t="n">
-        <v>31118.19</v>
+        <v>30913.19</v>
       </c>
       <c r="C68" s="5" t="n">
-        <v>30730</v>
+        <v>30525</v>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
@@ -6018,12 +5944,12 @@
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>-$210.78K</t>
+          <t>-$276.53K</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>+$348.43K</t>
+          <t>+$337.98K</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr">
@@ -6038,114 +5964,110 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="inlineStr">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B69" s="5" t="n">
-        <v>30913.19</v>
-      </c>
-      <c r="C69" s="5" t="n">
-        <v>30525</v>
-      </c>
-      <c r="D69" s="6" t="inlineStr">
+      <c r="B69" s="2" t="n">
+        <v>31108.19</v>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>30720</v>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E69" s="7" t="inlineStr">
-        <is>
-          <t>-$276.53K</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="inlineStr">
-        <is>
-          <t>+$337.98K</t>
-        </is>
-      </c>
-      <c r="G69" s="6" t="inlineStr">
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>-$68.83K</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>+$326.92K</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="n">
+        <v>31068.19</v>
+      </c>
+      <c r="C70" s="5" t="n">
+        <v>30680</v>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>-$223.68K</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>+$275.30K</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H69" s="6" t="inlineStr">
+      <c r="H70" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="3" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B70" s="2" t="n">
-        <v>31108.19</v>
-      </c>
-      <c r="C70" s="2" t="n">
-        <v>30720</v>
-      </c>
-      <c r="D70" s="3" t="inlineStr">
+      <c r="B71" s="2" t="n">
+        <v>31238.19</v>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>30850</v>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>-$68.83K</t>
-        </is>
-      </c>
-      <c r="F70" s="3" t="inlineStr">
-        <is>
-          <t>+$326.92K</t>
-        </is>
-      </c>
-      <c r="G70" s="3" t="inlineStr">
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>-$30.11K</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>+$262.40K</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H70" s="3" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="n">
-        <v>31068.19</v>
-      </c>
-      <c r="C71" s="5" t="n">
-        <v>30680</v>
-      </c>
-      <c r="D71" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E71" s="7" t="inlineStr">
-        <is>
-          <t>-$223.68K</t>
-        </is>
-      </c>
-      <c r="F71" s="6" t="inlineStr">
-        <is>
-          <t>+$275.30K</t>
-        </is>
-      </c>
-      <c r="G71" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H71" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
@@ -6154,24 +6076,24 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>31238.19</v>
+        <v>31263.19</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>30850</v>
+        <v>30875</v>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>-$30.11K</t>
+      <c r="E72" s="9" t="inlineStr">
+        <is>
+          <t>+$15.98K</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>+$262.40K</t>
+          <t>+$255.64K</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
@@ -6188,68 +6110,72 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>31263.19</v>
+        <v>31113.19</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>30875</v>
+        <v>30725</v>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E73" s="9" t="inlineStr">
-        <is>
-          <t>+$15.98K</t>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>-$51.62K</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>+$255.64K</t>
+          <t>+$223.68K</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H73" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="n">
-        <v>4095.53</v>
-      </c>
-      <c r="C74" s="2" t="n">
-        <v>369</v>
-      </c>
-      <c r="D74" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>-$172.93K</t>
-        </is>
-      </c>
-      <c r="F74" s="3" t="inlineStr">
-        <is>
-          <t>+$237.72K</t>
-        </is>
-      </c>
-      <c r="G74" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H74" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="n">
+        <v>30948.19</v>
+      </c>
+      <c r="C74" s="5" t="n">
+        <v>30560</v>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>-$209.55K</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>+$223.07K</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -6260,24 +6186,24 @@
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>31113.19</v>
+        <v>31168.19</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>30725</v>
+        <v>30780</v>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>-$51.62K</t>
+      <c r="E75" s="9" t="inlineStr">
+        <is>
+          <t>+$43.02K</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>+$223.68K</t>
+          <t>+$197.87K</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -6292,42 +6218,38 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="6" t="inlineStr">
+      <c r="A76" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B76" s="5" t="n">
-        <v>30948.19</v>
-      </c>
-      <c r="C76" s="5" t="n">
-        <v>30560</v>
-      </c>
-      <c r="D76" s="6" t="inlineStr">
+      <c r="B76" s="2" t="n">
+        <v>30968.19</v>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>30580</v>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E76" s="7" t="inlineStr">
-        <is>
-          <t>-$209.55K</t>
-        </is>
-      </c>
-      <c r="F76" s="6" t="inlineStr">
-        <is>
-          <t>+$223.07K</t>
-        </is>
-      </c>
-      <c r="G76" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H76" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>-$114.91K</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>+$135.19K</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -6336,10 +6258,10 @@
         </is>
       </c>
       <c r="B77" s="2" t="n">
-        <v>31168.19</v>
+        <v>31198.19</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>30780</v>
+        <v>30810</v>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
@@ -6348,12 +6270,12 @@
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>+$43.02K</t>
+          <t>+$77.43K</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>+$197.87K</t>
+          <t>+$129.05K</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -6374,10 +6296,10 @@
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>30968.19</v>
+        <v>31178.19</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>30580</v>
+        <v>30790</v>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
@@ -6386,20 +6308,24 @@
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>-$114.91K</t>
+          <t>-$81.73K</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>+$135.19K</t>
+          <t>+$124.75K</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H78" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -6408,24 +6334,24 @@
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>31198.19</v>
+        <v>31278.19</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>30810</v>
+        <v>30890</v>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E79" s="9" t="inlineStr">
-        <is>
-          <t>+$77.43K</t>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>-$67.90K</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>+$129.05K</t>
+          <t>+$123.83K</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -6435,7 +6361,7 @@
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -6446,10 +6372,10 @@
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>31178.19</v>
+        <v>31063.19</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>30790</v>
+        <v>30675</v>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
@@ -6458,12 +6384,12 @@
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>-$81.73K</t>
+          <t>-$25.81K</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>+$124.75K</t>
+          <t>+$68.83K</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -6473,7 +6399,7 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -6484,24 +6410,24 @@
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>31278.19</v>
+        <v>31013.19</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>30890</v>
+        <v>30625</v>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E81" s="4" t="inlineStr">
-        <is>
-          <t>-$67.90K</t>
+      <c r="E81" s="9" t="inlineStr">
+        <is>
+          <t>+$3.69K</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>+$123.83K</t>
+          <t>+$62.68K</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -6511,7 +6437,7 @@
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -6522,24 +6448,24 @@
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>31063.19</v>
+        <v>31078.19</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>30675</v>
+        <v>30690</v>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E82" s="4" t="inlineStr">
-        <is>
-          <t>-$25.81K</t>
+      <c r="E82" s="9" t="inlineStr">
+        <is>
+          <t>+$8.60K</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>+$68.83K</t>
+          <t>+$51.62K</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -6560,24 +6486,24 @@
         </is>
       </c>
       <c r="B83" s="2" t="n">
-        <v>31013.19</v>
+        <v>30958.19</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>30625</v>
+        <v>30570</v>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E83" s="9" t="inlineStr">
-        <is>
-          <t>+$3.69K</t>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>-$3.38K</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>+$62.68K</t>
+          <t>+$10.14K</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -6598,24 +6524,24 @@
         </is>
       </c>
       <c r="B84" s="2" t="n">
-        <v>31078.19</v>
+        <v>30918.19</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>30690</v>
+        <v>30530</v>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E84" s="9" t="inlineStr">
-        <is>
-          <t>+$8.60K</t>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>-$6.15K</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>+$51.62K</t>
+          <t>+$6.15K</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -6629,84 +6555,8 @@
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="n">
-        <v>30958.19</v>
-      </c>
-      <c r="C85" s="2" t="n">
-        <v>30570</v>
-      </c>
-      <c r="D85" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E85" s="4" t="inlineStr">
-        <is>
-          <t>-$3.38K</t>
-        </is>
-      </c>
-      <c r="F85" s="3" t="inlineStr">
-        <is>
-          <t>+$10.14K</t>
-        </is>
-      </c>
-      <c r="G85" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H85" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="n">
-        <v>30918.19</v>
-      </c>
-      <c r="C86" s="2" t="n">
-        <v>30530</v>
-      </c>
-      <c r="D86" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E86" s="4" t="inlineStr">
-        <is>
-          <t>-$6.15K</t>
-        </is>
-      </c>
-      <c r="F86" s="3" t="inlineStr">
-        <is>
-          <t>+$6.15K</t>
-        </is>
-      </c>
-      <c r="G86" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H86" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H86"/>
+  <autoFilter ref="A1:H84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>